<commit_message>
feat(meals): prepare Recipe persistence foundation
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/spec/meals/Meals Acceptance Checklist v1.0.xlsx
+++ b/spec/meals/Meals Acceptance Checklist v1.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wcoop\Documents\HomeMaintenanceApp\spec\meals\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7036922-060B-48E0-A57F-6D69BEA330D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F945ED1C-5F1E-4B5A-AB77-FEDF7CA21501}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5032" uniqueCount="1132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5056" uniqueCount="1137">
   <si>
     <t>Meals Acceptance Checklist</t>
   </si>
@@ -3547,6 +3547,21 @@
   </si>
   <si>
     <t>Phase 0A Meals foundation accepted. Live web routing, navigation, owner-auth integration, responsive shell, nested route refresh, and E2E-00 passed. Acceptance includes the Acceptance Workbook update tooling and Phase 0A release/deployment infrastructure. Recipe persistence, Recipe functionality beyond the Phase 0A shell/placeholders (including Add/Edit), Shopping functionality/persistence, meal-plan persistence, Weekly Planner meal integration, Recipe Import, future Meals database objects, and future Meals database-security/catalog verification remain outside this acceptance and are not yet accepted. Owner explicitly authorized this scope-limited acceptance on 2026-10-28 following P0-UAT-001.</t>
+  </si>
+  <si>
+    <t>P0B-PREFLIGHT-001</t>
+  </si>
+  <si>
+    <t>supabase/review/202610280001_meals_recipe_foundation.sql (disabled draft)</t>
+  </si>
+  <si>
+    <t>dev @ 75de46464a3b4eb5c72f4fadb9ac8c0baefde9d7; uncommitted reviewed draft</t>
+  </si>
+  <si>
+    <t>P0B-PREFLIGHT-001: meals-0b-production-preflight-manifest.json; complete catalog/supplement JSON and CSV evidence in session b7458d86-6190-4718-8779-7c2b79a30630/files; Dashboard-verified home-maintenance-app / tawvchmjtkgykwwvnnnn</t>
+  </si>
+  <si>
+    <t>P0B-PREFLIGHT-001 preflight-only: authenticated Dashboard identity, PostgreSQL 17.11, postgres object ownership/CREATE authority, browser-role safety, zero Meals collisions/dependencies and informational defaults captured. Canonical Category/Cuisine draft and local tests updated. No migration or production postflight executed; no database check marked Pass. Status Not Built and stage Both retained; post-deployment object ACL/RLS/owner and broker-independence checks remain required. Disabled reversal prepared, not executed. No Phase 0A UAT/acceptance or future owner decision changed.</t>
   </si>
 </sst>
 </file>
@@ -13875,8 +13890,10 @@
       </c>
       <c r="R2" s="2"/>
     </row>
-    <row r="3" spans="1:18" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="2"/>
+    <row r="3" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>1132</v>
+      </c>
       <c r="B3" s="2" t="s">
         <v>930</v>
       </c>
@@ -13889,15 +13906,21 @@
       <c r="E3" s="2" t="s">
         <v>814</v>
       </c>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
+      <c r="F3" s="2" t="s">
+        <v>1133</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>1134</v>
+      </c>
       <c r="H3" s="2" t="s">
         <v>926</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="J3" s="7"/>
+      <c r="J3" s="7" t="s">
+        <v>1130</v>
+      </c>
       <c r="K3" s="2" t="s">
         <v>927</v>
       </c>
@@ -13910,14 +13933,18 @@
       <c r="N3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="O3" s="2"/>
+      <c r="O3" s="2" t="s">
+        <v>1135</v>
+      </c>
       <c r="P3" s="2" t="s">
-        <v>929</v>
+        <v>927</v>
       </c>
       <c r="Q3" s="2" t="s">
         <v>929</v>
       </c>
-      <c r="R3" s="2"/>
+      <c r="R3" s="2" t="s">
+        <v>1136</v>
+      </c>
     </row>
     <row r="4" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
@@ -14051,8 +14078,10 @@
       </c>
       <c r="R6" s="2"/>
     </row>
-    <row r="7" spans="1:18" ht="45" x14ac:dyDescent="0.25">
-      <c r="A7" s="2"/>
+    <row r="7" spans="1:18" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>1132</v>
+      </c>
       <c r="B7" s="2" t="s">
         <v>936</v>
       </c>
@@ -14065,15 +14094,21 @@
       <c r="E7" s="2" t="s">
         <v>814</v>
       </c>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
+      <c r="F7" s="2" t="s">
+        <v>1133</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>1134</v>
+      </c>
       <c r="H7" s="2" t="s">
         <v>926</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="J7" s="7"/>
+      <c r="J7" s="7" t="s">
+        <v>1130</v>
+      </c>
       <c r="K7" s="2" t="s">
         <v>929</v>
       </c>
@@ -14086,14 +14121,18 @@
       <c r="N7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="O7" s="2"/>
+      <c r="O7" s="2" t="s">
+        <v>1135</v>
+      </c>
       <c r="P7" s="2" t="s">
-        <v>929</v>
+        <v>927</v>
       </c>
       <c r="Q7" s="2" t="s">
         <v>929</v>
       </c>
-      <c r="R7" s="2"/>
+      <c r="R7" s="2" t="s">
+        <v>1136</v>
+      </c>
     </row>
     <row r="8" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
@@ -14667,8 +14706,10 @@
       </c>
       <c r="R20" s="2"/>
     </row>
-    <row r="21" spans="1:18" ht="30" x14ac:dyDescent="0.25">
-      <c r="A21" s="2"/>
+    <row r="21" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>1132</v>
+      </c>
       <c r="B21" s="2" t="s">
         <v>979</v>
       </c>
@@ -14681,15 +14722,21 @@
       <c r="E21" s="2" t="s">
         <v>980</v>
       </c>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
+      <c r="F21" s="2" t="s">
+        <v>1133</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>1134</v>
+      </c>
       <c r="H21" s="2" t="s">
         <v>926</v>
       </c>
       <c r="I21" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="J21" s="7"/>
+      <c r="J21" s="7" t="s">
+        <v>1130</v>
+      </c>
       <c r="K21" s="2" t="s">
         <v>927</v>
       </c>
@@ -14702,17 +14749,23 @@
       <c r="N21" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="O21" s="2"/>
+      <c r="O21" s="2" t="s">
+        <v>1135</v>
+      </c>
       <c r="P21" s="2" t="s">
-        <v>929</v>
+        <v>927</v>
       </c>
       <c r="Q21" s="2" t="s">
         <v>929</v>
       </c>
-      <c r="R21" s="2"/>
-    </row>
-    <row r="22" spans="1:18" ht="45" x14ac:dyDescent="0.25">
-      <c r="A22" s="2"/>
+      <c r="R21" s="2" t="s">
+        <v>1136</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>1132</v>
+      </c>
       <c r="B22" s="2" t="s">
         <v>983</v>
       </c>
@@ -14725,15 +14778,21 @@
       <c r="E22" s="2" t="s">
         <v>984</v>
       </c>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
+      <c r="F22" s="2" t="s">
+        <v>1133</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>1134</v>
+      </c>
       <c r="H22" s="2" t="s">
         <v>926</v>
       </c>
       <c r="I22" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="J22" s="7"/>
+      <c r="J22" s="7" t="s">
+        <v>1130</v>
+      </c>
       <c r="K22" s="2" t="s">
         <v>929</v>
       </c>
@@ -14746,14 +14805,18 @@
       <c r="N22" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="O22" s="2"/>
+      <c r="O22" s="2" t="s">
+        <v>1135</v>
+      </c>
       <c r="P22" s="2" t="s">
-        <v>929</v>
+        <v>927</v>
       </c>
       <c r="Q22" s="2" t="s">
         <v>929</v>
       </c>
-      <c r="R22" s="2"/>
+      <c r="R22" s="2" t="s">
+        <v>1136</v>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="G2:G22">
@@ -16190,14 +16253,14 @@
         <f>IFERROR(INDEX('Database Verification'!$N:$N,MATCH($I16,'Database Verification'!$B:$B,0)),"")</f>
         <v>Not Built</v>
       </c>
-      <c r="K16" s="7">
+      <c r="K16" s="7" t="str">
         <f>IFERROR(INDEX('Database Verification'!$J:$J,MATCH($I16,'Database Verification'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>2026-10-28</v>
       </c>
       <c r="L16" s="2"/>
-      <c r="M16" s="2">
+      <c r="M16" s="2" t="str">
         <f>IFERROR(INDEX('Database Verification'!$O:$O,MATCH($I16,'Database Verification'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P0B-PREFLIGHT-001: meals-0b-production-preflight-manifest.json; complete catalog/supplement JSON and CSV evidence in session b7458d86-6190-4718-8779-7c2b79a30630/files; Dashboard-verified home-maintenance-app / tawvchmjtkgykwwvnnnn</v>
       </c>
       <c r="N16" s="2" t="s">
         <v>1075</v>

</xml_diff>

<commit_message>
feat(meals): implement Phase 1 Recipe Core
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/spec/meals/Meals Acceptance Checklist v1.0.xlsx
+++ b/spec/meals/Meals Acceptance Checklist v1.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wcoop\Documents\HomeMaintenanceApp\spec\meals\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02963D1F-5BC3-40A9-A86C-51F6B2392F42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91417126-1D94-4337-8CEA-D4028A336DE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5134" uniqueCount="1155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5376" uniqueCount="1161">
   <si>
     <t>Meals Acceptance Checklist</t>
   </si>
@@ -3621,6 +3621,24 @@
   </si>
   <si>
     <t>P0B-DB-001 Recipe foundation scope only. Captured production catalog and synthetic SQL SET ROLE/claim evidence, not live JWT/API authentication, owner application UAT or Recipe UI evidence. Future Meals objects require their own verification. No deployment blocker observed; blocker classification field is unchanged. Reversal prepared, not executed; test-only transaction rollback is not migration reversal. Production postflight effective_anon_denial/explicit_table_acl/function_acl/column_acl passed.</t>
+  </si>
+  <si>
+    <t>Local Recipe Core implementation and technical checks complete. Isolated browser/handler/PGlite evidence only; not live owner JWT/API or owner UAT. Await authorized deployment and independent owner desktop/mobile verification. Phase 2/3 actions remain unavailable.</t>
+  </si>
+  <si>
+    <t>P1-TECH-001</t>
+  </si>
+  <si>
+    <t>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</t>
+  </si>
+  <si>
+    <t>Prepared with deterministic run-prefixed IDs and Recipe-before-lookup cleanup in spec/meals/README.md. Local synthetic flow exercised and fixture counts returned to zero. Live owner E2E/UAT remains unexecuted pending authorized deployment. No Shopping/Planner data created.</t>
+  </si>
+  <si>
+    <t>Recipe UI/service ready for post-release owner/API checks. Local source/build, isolated synthetic browser and exact-migration PGlite role tests passed. These do not prove live JWT/PostgREST authorization; composite application/API verification is not marked Pass. Prior production P0B evidence is unchanged.</t>
+  </si>
+  <si>
+    <t>Executed local source/build inspection and unchanged-migration PGlite catalog tests: direct table service, no application-callable Recipe RPC/function and no SECURITY DEFINER introduced. Existing internal trigger remains invoker and not browser-callable. Local technical scope only, not owner application/API authentication proof.</t>
   </si>
 </sst>
 </file>
@@ -4881,11 +4899,11 @@
       </c>
       <c r="G7" s="5">
         <f>COUNTIF('Functional Acceptance'!$L:$L,"Ready to Test")</f>
-        <v>0</v>
+        <v>68</v>
       </c>
       <c r="H7" s="5">
         <f>COUNTIF('Functional Acceptance'!$L:$L,"Not Built")</f>
-        <v>166</v>
+        <v>98</v>
       </c>
       <c r="I7" s="5">
         <f>COUNTIF('Functional Acceptance'!$L:$L,"Deferred")</f>
@@ -4918,11 +4936,11 @@
       </c>
       <c r="G8" s="5">
         <f>COUNTIF('End-to-End Tests'!$J:$J,"Ready to Test")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H8" s="5">
         <f>COUNTIF('End-to-End Tests'!$J:$J,"Not Built")</f>
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="I8" s="5">
         <f>COUNTIF('End-to-End Tests'!$J:$J,"Deferred")</f>
@@ -4939,7 +4957,7 @@
       </c>
       <c r="C9" s="5">
         <f>COUNTIF('Security Acceptance'!$N:$N,"Pass")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D9" s="5">
         <f>COUNTIF('Security Acceptance'!$N:$N,"Pass with Known Issue")</f>
@@ -4955,11 +4973,11 @@
       </c>
       <c r="G9" s="5">
         <f>COUNTIF('Security Acceptance'!$N:$N,"Ready to Test")</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H9" s="5">
         <f>COUNTIF('Security Acceptance'!$N:$N,"Not Built")</f>
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="I9" s="5">
         <f>COUNTIF('Security Acceptance'!$N:$N,"Deferred")</f>
@@ -5212,7 +5230,7 @@
       </c>
       <c r="E23" s="2">
         <f>COUNTIFS('Functional Acceptance'!D:D,A23,'Functional Acceptance'!L:L,"Pass")+COUNTIFS('Security Acceptance'!D:D,A23,'Security Acceptance'!N:N,"Pass")+COUNTIFS('Database Verification'!D:D,A23,'Database Verification'!N:N,"Pass")+COUNTIFS('End-to-End Tests'!C:C,A23,'End-to-End Tests'!J:J,"Pass")</f>
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F23" s="2">
         <f>COUNTIFS('Functional Acceptance'!D:D,A23,'Functional Acceptance'!L:L,"Pass with Known Issue")+COUNTIFS('Security Acceptance'!D:D,A23,'Security Acceptance'!N:N,"Pass with Known Issue")+COUNTIFS('Database Verification'!D:D,A23,'Database Verification'!N:N,"Pass with Known Issue")+COUNTIFS('End-to-End Tests'!C:C,A23,'End-to-End Tests'!J:J,"Pass with Known Issue")</f>
@@ -5758,7 +5776,9 @@
       </c>
     </row>
     <row r="6" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="2"/>
+      <c r="A6" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B6" s="2" t="s">
         <v>116</v>
       </c>
@@ -5790,15 +5810,21 @@
         <v>119</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M6" s="7"/>
       <c r="N6" s="2"/>
-      <c r="O6" s="2"/>
-      <c r="P6" s="2"/>
+      <c r="O6" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P6" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="7" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="2"/>
+      <c r="A7" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B7" s="2" t="s">
         <v>120</v>
       </c>
@@ -5830,12 +5856,16 @@
         <v>123</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M7" s="7"/>
       <c r="N7" s="2"/>
-      <c r="O7" s="2"/>
-      <c r="P7" s="2"/>
+      <c r="O7" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P7" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="8" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
@@ -5926,7 +5956,9 @@
       </c>
     </row>
     <row r="10" spans="1:16" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="2"/>
+      <c r="A10" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B10" s="2" t="s">
         <v>132</v>
       </c>
@@ -5958,15 +5990,21 @@
         <v>139</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M10" s="7"/>
       <c r="N10" s="2"/>
-      <c r="O10" s="2"/>
-      <c r="P10" s="2"/>
+      <c r="O10" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P10" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="11" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="2"/>
+      <c r="A11" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B11" s="2" t="s">
         <v>140</v>
       </c>
@@ -5998,15 +6036,21 @@
         <v>139</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M11" s="7"/>
       <c r="N11" s="2"/>
-      <c r="O11" s="2"/>
-      <c r="P11" s="2"/>
+      <c r="O11" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P11" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="12" spans="1:16" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="2"/>
+      <c r="A12" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B12" s="2" t="s">
         <v>143</v>
       </c>
@@ -6038,15 +6082,21 @@
         <v>146</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M12" s="7"/>
       <c r="N12" s="2"/>
-      <c r="O12" s="2"/>
-      <c r="P12" s="2"/>
+      <c r="O12" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P12" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="13" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="2"/>
+      <c r="A13" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B13" s="2" t="s">
         <v>147</v>
       </c>
@@ -6078,15 +6128,21 @@
         <v>150</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M13" s="7"/>
       <c r="N13" s="2"/>
-      <c r="O13" s="2"/>
-      <c r="P13" s="2"/>
+      <c r="O13" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P13" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="14" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="2"/>
+      <c r="A14" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B14" s="2" t="s">
         <v>151</v>
       </c>
@@ -6118,15 +6174,21 @@
         <v>154</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M14" s="7"/>
       <c r="N14" s="2"/>
-      <c r="O14" s="2"/>
-      <c r="P14" s="2"/>
+      <c r="O14" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P14" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="15" spans="1:16" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="2"/>
+      <c r="A15" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B15" s="2" t="s">
         <v>155</v>
       </c>
@@ -6158,15 +6220,21 @@
         <v>159</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M15" s="7"/>
       <c r="N15" s="2"/>
-      <c r="O15" s="2"/>
-      <c r="P15" s="2"/>
+      <c r="O15" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P15" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="16" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="2"/>
+      <c r="A16" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B16" s="2" t="s">
         <v>160</v>
       </c>
@@ -6198,15 +6266,21 @@
         <v>164</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M16" s="7"/>
       <c r="N16" s="2"/>
-      <c r="O16" s="2"/>
-      <c r="P16" s="2"/>
+      <c r="O16" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P16" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="17" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="2"/>
+      <c r="A17" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B17" s="2" t="s">
         <v>165</v>
       </c>
@@ -6238,15 +6312,21 @@
         <v>168</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M17" s="7"/>
       <c r="N17" s="2"/>
-      <c r="O17" s="2"/>
-      <c r="P17" s="2"/>
+      <c r="O17" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P17" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="18" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="2"/>
+      <c r="A18" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B18" s="2" t="s">
         <v>169</v>
       </c>
@@ -6278,15 +6358,21 @@
         <v>172</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M18" s="7"/>
       <c r="N18" s="2"/>
-      <c r="O18" s="2"/>
-      <c r="P18" s="2"/>
+      <c r="O18" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P18" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="19" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="2"/>
+      <c r="A19" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B19" s="2" t="s">
         <v>173</v>
       </c>
@@ -6318,15 +6404,21 @@
         <v>176</v>
       </c>
       <c r="L19" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M19" s="7"/>
       <c r="N19" s="2"/>
-      <c r="O19" s="2"/>
-      <c r="P19" s="2"/>
+      <c r="O19" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P19" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="20" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="2"/>
+      <c r="A20" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B20" s="2" t="s">
         <v>177</v>
       </c>
@@ -6358,15 +6450,21 @@
         <v>180</v>
       </c>
       <c r="L20" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M20" s="7"/>
       <c r="N20" s="2"/>
-      <c r="O20" s="2"/>
-      <c r="P20" s="2"/>
+      <c r="O20" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P20" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="21" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="2"/>
+      <c r="A21" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B21" s="2" t="s">
         <v>181</v>
       </c>
@@ -6398,15 +6496,21 @@
         <v>184</v>
       </c>
       <c r="L21" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M21" s="7"/>
       <c r="N21" s="2"/>
-      <c r="O21" s="2"/>
-      <c r="P21" s="2"/>
+      <c r="O21" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P21" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="22" spans="1:16" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="2"/>
+      <c r="A22" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B22" s="2" t="s">
         <v>185</v>
       </c>
@@ -6438,15 +6542,21 @@
         <v>189</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M22" s="7"/>
       <c r="N22" s="2"/>
-      <c r="O22" s="2"/>
-      <c r="P22" s="2"/>
+      <c r="O22" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P22" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="23" spans="1:16" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="2"/>
+      <c r="A23" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B23" s="2" t="s">
         <v>190</v>
       </c>
@@ -6478,15 +6588,21 @@
         <v>189</v>
       </c>
       <c r="L23" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M23" s="7"/>
       <c r="N23" s="2"/>
-      <c r="O23" s="2"/>
-      <c r="P23" s="2"/>
+      <c r="O23" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P23" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="24" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="2"/>
+      <c r="A24" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B24" s="2" t="s">
         <v>191</v>
       </c>
@@ -6518,15 +6634,21 @@
         <v>194</v>
       </c>
       <c r="L24" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M24" s="7"/>
       <c r="N24" s="2"/>
-      <c r="O24" s="2"/>
-      <c r="P24" s="2"/>
+      <c r="O24" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P24" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="25" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="2"/>
+      <c r="A25" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B25" s="2" t="s">
         <v>195</v>
       </c>
@@ -6558,15 +6680,21 @@
         <v>198</v>
       </c>
       <c r="L25" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M25" s="7"/>
       <c r="N25" s="2"/>
-      <c r="O25" s="2"/>
-      <c r="P25" s="2"/>
+      <c r="O25" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P25" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="26" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="2"/>
+      <c r="A26" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B26" s="2" t="s">
         <v>199</v>
       </c>
@@ -6598,12 +6726,16 @@
         <v>202</v>
       </c>
       <c r="L26" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M26" s="7"/>
       <c r="N26" s="2"/>
-      <c r="O26" s="2"/>
-      <c r="P26" s="2"/>
+      <c r="O26" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P26" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="27" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
@@ -6726,7 +6858,9 @@
       <c r="P29" s="2"/>
     </row>
     <row r="30" spans="1:16" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="2"/>
+      <c r="A30" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B30" s="2" t="s">
         <v>215</v>
       </c>
@@ -6758,15 +6892,21 @@
         <v>218</v>
       </c>
       <c r="L30" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M30" s="7"/>
       <c r="N30" s="2"/>
-      <c r="O30" s="2"/>
-      <c r="P30" s="2"/>
+      <c r="O30" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P30" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="31" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="2"/>
+      <c r="A31" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B31" s="2" t="s">
         <v>219</v>
       </c>
@@ -6798,15 +6938,21 @@
         <v>222</v>
       </c>
       <c r="L31" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M31" s="7"/>
       <c r="N31" s="2"/>
-      <c r="O31" s="2"/>
-      <c r="P31" s="2"/>
+      <c r="O31" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P31" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="32" spans="1:16" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="2"/>
+      <c r="A32" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B32" s="2" t="s">
         <v>223</v>
       </c>
@@ -6838,15 +6984,21 @@
         <v>227</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M32" s="7"/>
       <c r="N32" s="2"/>
-      <c r="O32" s="2"/>
-      <c r="P32" s="2"/>
+      <c r="O32" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P32" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="33" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="2"/>
+      <c r="A33" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B33" s="2" t="s">
         <v>228</v>
       </c>
@@ -6878,15 +7030,21 @@
         <v>231</v>
       </c>
       <c r="L33" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M33" s="7"/>
       <c r="N33" s="2"/>
-      <c r="O33" s="2"/>
-      <c r="P33" s="2"/>
+      <c r="O33" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P33" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="34" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="2"/>
+      <c r="A34" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B34" s="2" t="s">
         <v>232</v>
       </c>
@@ -6918,15 +7076,21 @@
         <v>236</v>
       </c>
       <c r="L34" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M34" s="7"/>
       <c r="N34" s="2"/>
-      <c r="O34" s="2"/>
-      <c r="P34" s="2"/>
+      <c r="O34" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P34" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="35" spans="1:16" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="2"/>
+      <c r="A35" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B35" s="2" t="s">
         <v>237</v>
       </c>
@@ -6958,12 +7122,16 @@
         <v>240</v>
       </c>
       <c r="L35" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M35" s="7"/>
       <c r="N35" s="2"/>
-      <c r="O35" s="2"/>
-      <c r="P35" s="2"/>
+      <c r="O35" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P35" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="36" spans="1:16" ht="105" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2"/>
@@ -7006,7 +7174,9 @@
       <c r="P36" s="2"/>
     </row>
     <row r="37" spans="1:16" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="2"/>
+      <c r="A37" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B37" s="2" t="s">
         <v>245</v>
       </c>
@@ -7038,15 +7208,21 @@
         <v>249</v>
       </c>
       <c r="L37" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M37" s="7"/>
       <c r="N37" s="2"/>
-      <c r="O37" s="2"/>
-      <c r="P37" s="2"/>
+      <c r="O37" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P37" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="38" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="2"/>
+      <c r="A38" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B38" s="2" t="s">
         <v>250</v>
       </c>
@@ -7078,15 +7254,21 @@
         <v>249</v>
       </c>
       <c r="L38" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M38" s="7"/>
       <c r="N38" s="2"/>
-      <c r="O38" s="2"/>
-      <c r="P38" s="2"/>
+      <c r="O38" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P38" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="39" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="2"/>
+      <c r="A39" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B39" s="2" t="s">
         <v>251</v>
       </c>
@@ -7118,15 +7300,21 @@
         <v>254</v>
       </c>
       <c r="L39" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M39" s="7"/>
       <c r="N39" s="2"/>
-      <c r="O39" s="2"/>
-      <c r="P39" s="2"/>
+      <c r="O39" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P39" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="40" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="2"/>
+      <c r="A40" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B40" s="2" t="s">
         <v>255</v>
       </c>
@@ -7158,15 +7346,21 @@
         <v>258</v>
       </c>
       <c r="L40" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M40" s="7"/>
       <c r="N40" s="2"/>
-      <c r="O40" s="2"/>
-      <c r="P40" s="2"/>
+      <c r="O40" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P40" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="41" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="2"/>
+      <c r="A41" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B41" s="2" t="s">
         <v>259</v>
       </c>
@@ -7198,12 +7392,16 @@
         <v>262</v>
       </c>
       <c r="L41" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M41" s="7"/>
       <c r="N41" s="2"/>
-      <c r="O41" s="2"/>
-      <c r="P41" s="2"/>
+      <c r="O41" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P41" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="42" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="2"/>
@@ -7286,7 +7484,9 @@
       <c r="P43" s="2"/>
     </row>
     <row r="44" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="2"/>
+      <c r="A44" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B44" s="2" t="s">
         <v>271</v>
       </c>
@@ -7318,15 +7518,21 @@
         <v>274</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M44" s="7"/>
       <c r="N44" s="2"/>
-      <c r="O44" s="2"/>
-      <c r="P44" s="2"/>
+      <c r="O44" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P44" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="45" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="2"/>
+      <c r="A45" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B45" s="2" t="s">
         <v>275</v>
       </c>
@@ -7358,15 +7564,21 @@
         <v>278</v>
       </c>
       <c r="L45" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M45" s="7"/>
       <c r="N45" s="2"/>
-      <c r="O45" s="2"/>
-      <c r="P45" s="2"/>
+      <c r="O45" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P45" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="46" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="2"/>
+      <c r="A46" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B46" s="2" t="s">
         <v>279</v>
       </c>
@@ -7398,15 +7610,21 @@
         <v>282</v>
       </c>
       <c r="L46" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M46" s="7"/>
       <c r="N46" s="2"/>
-      <c r="O46" s="2"/>
-      <c r="P46" s="2"/>
+      <c r="O46" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P46" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="47" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="2"/>
+      <c r="A47" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B47" s="2" t="s">
         <v>283</v>
       </c>
@@ -7438,12 +7656,16 @@
         <v>286</v>
       </c>
       <c r="L47" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M47" s="7"/>
       <c r="N47" s="2"/>
-      <c r="O47" s="2"/>
-      <c r="P47" s="2"/>
+      <c r="O47" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P47" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="48" spans="1:16" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="2"/>
@@ -7526,7 +7748,9 @@
       <c r="P49" s="2"/>
     </row>
     <row r="50" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="2"/>
+      <c r="A50" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B50" s="2" t="s">
         <v>295</v>
       </c>
@@ -7558,15 +7782,21 @@
         <v>299</v>
       </c>
       <c r="L50" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M50" s="7"/>
       <c r="N50" s="2"/>
-      <c r="O50" s="2"/>
-      <c r="P50" s="2"/>
+      <c r="O50" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P50" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="51" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="2"/>
+      <c r="A51" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B51" s="2" t="s">
         <v>300</v>
       </c>
@@ -7598,15 +7828,21 @@
         <v>304</v>
       </c>
       <c r="L51" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M51" s="7"/>
       <c r="N51" s="2"/>
-      <c r="O51" s="2"/>
-      <c r="P51" s="2"/>
+      <c r="O51" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P51" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="52" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="2"/>
+      <c r="A52" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B52" s="2" t="s">
         <v>305</v>
       </c>
@@ -7638,15 +7874,21 @@
         <v>308</v>
       </c>
       <c r="L52" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M52" s="7"/>
       <c r="N52" s="2"/>
-      <c r="O52" s="2"/>
-      <c r="P52" s="2"/>
+      <c r="O52" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P52" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="53" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="2"/>
+      <c r="A53" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B53" s="2" t="s">
         <v>309</v>
       </c>
@@ -7678,15 +7920,21 @@
         <v>312</v>
       </c>
       <c r="L53" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M53" s="7"/>
       <c r="N53" s="2"/>
-      <c r="O53" s="2"/>
-      <c r="P53" s="2"/>
+      <c r="O53" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P53" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="54" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="2"/>
+      <c r="A54" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B54" s="2" t="s">
         <v>313</v>
       </c>
@@ -7718,15 +7966,21 @@
         <v>316</v>
       </c>
       <c r="L54" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M54" s="7"/>
       <c r="N54" s="2"/>
-      <c r="O54" s="2"/>
-      <c r="P54" s="2"/>
+      <c r="O54" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P54" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="55" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="2"/>
+      <c r="A55" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B55" s="2" t="s">
         <v>317</v>
       </c>
@@ -7758,15 +8012,21 @@
         <v>320</v>
       </c>
       <c r="L55" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M55" s="7"/>
       <c r="N55" s="2"/>
-      <c r="O55" s="2"/>
-      <c r="P55" s="2"/>
+      <c r="O55" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P55" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="56" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="2"/>
+      <c r="A56" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B56" s="2" t="s">
         <v>321</v>
       </c>
@@ -7798,15 +8058,21 @@
         <v>324</v>
       </c>
       <c r="L56" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M56" s="7"/>
       <c r="N56" s="2"/>
-      <c r="O56" s="2"/>
-      <c r="P56" s="2"/>
+      <c r="O56" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P56" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="57" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="2"/>
+      <c r="A57" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B57" s="2" t="s">
         <v>325</v>
       </c>
@@ -7838,15 +8104,21 @@
         <v>328</v>
       </c>
       <c r="L57" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M57" s="7"/>
       <c r="N57" s="2"/>
-      <c r="O57" s="2"/>
-      <c r="P57" s="2"/>
+      <c r="O57" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P57" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="58" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="2"/>
+      <c r="A58" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B58" s="2" t="s">
         <v>329</v>
       </c>
@@ -7878,15 +8150,21 @@
         <v>332</v>
       </c>
       <c r="L58" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M58" s="7"/>
       <c r="N58" s="2"/>
-      <c r="O58" s="2"/>
-      <c r="P58" s="2"/>
+      <c r="O58" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P58" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="59" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="2"/>
+      <c r="A59" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B59" s="2" t="s">
         <v>333</v>
       </c>
@@ -7918,15 +8196,21 @@
         <v>336</v>
       </c>
       <c r="L59" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M59" s="7"/>
       <c r="N59" s="2"/>
-      <c r="O59" s="2"/>
-      <c r="P59" s="2"/>
+      <c r="O59" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P59" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="60" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="2"/>
+      <c r="A60" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B60" s="2" t="s">
         <v>337</v>
       </c>
@@ -7958,15 +8242,21 @@
         <v>340</v>
       </c>
       <c r="L60" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M60" s="7"/>
       <c r="N60" s="2"/>
-      <c r="O60" s="2"/>
-      <c r="P60" s="2"/>
+      <c r="O60" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P60" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="61" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="2"/>
+      <c r="A61" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B61" s="2" t="s">
         <v>341</v>
       </c>
@@ -7998,15 +8288,21 @@
         <v>344</v>
       </c>
       <c r="L61" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M61" s="7"/>
       <c r="N61" s="2"/>
-      <c r="O61" s="2"/>
-      <c r="P61" s="2"/>
+      <c r="O61" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P61" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="62" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="2"/>
+      <c r="A62" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B62" s="2" t="s">
         <v>345</v>
       </c>
@@ -8038,15 +8334,21 @@
         <v>349</v>
       </c>
       <c r="L62" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M62" s="7"/>
       <c r="N62" s="2"/>
-      <c r="O62" s="2"/>
-      <c r="P62" s="2"/>
+      <c r="O62" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P62" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="63" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="2"/>
+      <c r="A63" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B63" s="2" t="s">
         <v>350</v>
       </c>
@@ -8078,15 +8380,21 @@
         <v>353</v>
       </c>
       <c r="L63" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M63" s="7"/>
       <c r="N63" s="2"/>
-      <c r="O63" s="2"/>
-      <c r="P63" s="2"/>
+      <c r="O63" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P63" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="64" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="2"/>
+      <c r="A64" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B64" s="2" t="s">
         <v>354</v>
       </c>
@@ -8118,15 +8426,21 @@
         <v>357</v>
       </c>
       <c r="L64" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M64" s="7"/>
       <c r="N64" s="2"/>
-      <c r="O64" s="2"/>
-      <c r="P64" s="2"/>
+      <c r="O64" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P64" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="65" spans="1:16" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="2"/>
+      <c r="A65" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B65" s="2" t="s">
         <v>358</v>
       </c>
@@ -8158,15 +8472,21 @@
         <v>361</v>
       </c>
       <c r="L65" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M65" s="7"/>
       <c r="N65" s="2"/>
-      <c r="O65" s="2"/>
-      <c r="P65" s="2"/>
+      <c r="O65" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P65" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="66" spans="1:16" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="2"/>
+      <c r="A66" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B66" s="2" t="s">
         <v>362</v>
       </c>
@@ -8198,15 +8518,21 @@
         <v>365</v>
       </c>
       <c r="L66" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M66" s="7"/>
       <c r="N66" s="2"/>
-      <c r="O66" s="2"/>
-      <c r="P66" s="2"/>
+      <c r="O66" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P66" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="67" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="2"/>
+      <c r="A67" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B67" s="2" t="s">
         <v>366</v>
       </c>
@@ -8238,15 +8564,21 @@
         <v>365</v>
       </c>
       <c r="L67" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M67" s="7"/>
       <c r="N67" s="2"/>
-      <c r="O67" s="2"/>
-      <c r="P67" s="2"/>
+      <c r="O67" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P67" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="68" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="2"/>
+      <c r="A68" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B68" s="2" t="s">
         <v>367</v>
       </c>
@@ -8278,15 +8610,21 @@
         <v>370</v>
       </c>
       <c r="L68" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M68" s="7"/>
       <c r="N68" s="2"/>
-      <c r="O68" s="2"/>
-      <c r="P68" s="2"/>
+      <c r="O68" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P68" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="69" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="2"/>
+      <c r="A69" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B69" s="2" t="s">
         <v>371</v>
       </c>
@@ -8318,15 +8656,21 @@
         <v>375</v>
       </c>
       <c r="L69" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M69" s="7"/>
       <c r="N69" s="2"/>
-      <c r="O69" s="2"/>
-      <c r="P69" s="2"/>
+      <c r="O69" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P69" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="70" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="2"/>
+      <c r="A70" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B70" s="2" t="s">
         <v>376</v>
       </c>
@@ -8358,15 +8702,21 @@
         <v>379</v>
       </c>
       <c r="L70" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M70" s="7"/>
       <c r="N70" s="2"/>
-      <c r="O70" s="2"/>
-      <c r="P70" s="2"/>
+      <c r="O70" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P70" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="71" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="2"/>
+      <c r="A71" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B71" s="2" t="s">
         <v>380</v>
       </c>
@@ -8398,15 +8748,21 @@
         <v>384</v>
       </c>
       <c r="L71" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M71" s="7"/>
       <c r="N71" s="2"/>
-      <c r="O71" s="2"/>
-      <c r="P71" s="2"/>
+      <c r="O71" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P71" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="72" spans="1:16" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="2"/>
+      <c r="A72" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B72" s="2" t="s">
         <v>385</v>
       </c>
@@ -8438,15 +8794,21 @@
         <v>389</v>
       </c>
       <c r="L72" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M72" s="7"/>
       <c r="N72" s="2"/>
-      <c r="O72" s="2"/>
-      <c r="P72" s="2"/>
+      <c r="O72" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P72" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="73" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="2"/>
+      <c r="A73" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B73" s="2" t="s">
         <v>390</v>
       </c>
@@ -8478,15 +8840,21 @@
         <v>393</v>
       </c>
       <c r="L73" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M73" s="7"/>
       <c r="N73" s="2"/>
-      <c r="O73" s="2"/>
-      <c r="P73" s="2"/>
+      <c r="O73" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P73" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="74" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="2"/>
+      <c r="A74" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B74" s="2" t="s">
         <v>394</v>
       </c>
@@ -8518,12 +8886,16 @@
         <v>397</v>
       </c>
       <c r="L74" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M74" s="7"/>
       <c r="N74" s="2"/>
-      <c r="O74" s="2"/>
-      <c r="P74" s="2"/>
+      <c r="O74" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P74" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="75" spans="1:16" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="2"/>
@@ -12142,7 +12514,9 @@
       </c>
     </row>
     <row r="165" spans="1:16" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A165" s="2"/>
+      <c r="A165" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B165" s="2" t="s">
         <v>772</v>
       </c>
@@ -12174,15 +12548,21 @@
         <v>775</v>
       </c>
       <c r="L165" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M165" s="7"/>
       <c r="N165" s="2"/>
-      <c r="O165" s="2"/>
-      <c r="P165" s="2"/>
+      <c r="O165" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P165" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="166" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A166" s="2"/>
+      <c r="A166" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B166" s="2" t="s">
         <v>776</v>
       </c>
@@ -12214,15 +12594,21 @@
         <v>779</v>
       </c>
       <c r="L166" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M166" s="7"/>
       <c r="N166" s="2"/>
-      <c r="O166" s="2"/>
-      <c r="P166" s="2"/>
+      <c r="O166" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P166" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="167" spans="1:16" ht="105" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A167" s="2"/>
+      <c r="A167" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B167" s="2" t="s">
         <v>780</v>
       </c>
@@ -12254,15 +12640,21 @@
         <v>784</v>
       </c>
       <c r="L167" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M167" s="7"/>
       <c r="N167" s="2"/>
-      <c r="O167" s="2"/>
-      <c r="P167" s="2"/>
+      <c r="O167" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P167" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="168" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A168" s="2"/>
+      <c r="A168" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B168" s="2" t="s">
         <v>785</v>
       </c>
@@ -12294,15 +12686,21 @@
         <v>788</v>
       </c>
       <c r="L168" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M168" s="7"/>
       <c r="N168" s="2"/>
-      <c r="O168" s="2"/>
-      <c r="P168" s="2"/>
+      <c r="O168" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P168" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="169" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A169" s="2"/>
+      <c r="A169" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B169" s="2" t="s">
         <v>789</v>
       </c>
@@ -12334,15 +12732,21 @@
         <v>792</v>
       </c>
       <c r="L169" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M169" s="7"/>
       <c r="N169" s="2"/>
-      <c r="O169" s="2"/>
-      <c r="P169" s="2"/>
+      <c r="O169" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P169" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="170" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A170" s="2"/>
+      <c r="A170" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B170" s="2" t="s">
         <v>793</v>
       </c>
@@ -12374,15 +12778,21 @@
         <v>796</v>
       </c>
       <c r="L170" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M170" s="7"/>
       <c r="N170" s="2"/>
-      <c r="O170" s="2"/>
-      <c r="P170" s="2"/>
+      <c r="O170" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P170" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="171" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A171" s="2"/>
+      <c r="A171" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B171" s="2" t="s">
         <v>797</v>
       </c>
@@ -12414,15 +12824,21 @@
         <v>796</v>
       </c>
       <c r="L171" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M171" s="7"/>
       <c r="N171" s="2"/>
-      <c r="O171" s="2"/>
-      <c r="P171" s="2"/>
+      <c r="O171" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P171" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="172" spans="1:16" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A172" s="2"/>
+      <c r="A172" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B172" s="2" t="s">
         <v>798</v>
       </c>
@@ -12454,12 +12870,16 @@
         <v>801</v>
       </c>
       <c r="L172" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M172" s="7"/>
       <c r="N172" s="2"/>
-      <c r="O172" s="2"/>
-      <c r="P172" s="2"/>
+      <c r="O172" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P172" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
     <row r="173" spans="1:16" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A173" s="2"/>
@@ -12502,7 +12922,9 @@
       <c r="P173" s="2"/>
     </row>
     <row r="174" spans="1:16" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A174" s="2"/>
+      <c r="A174" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B174" s="2" t="s">
         <v>806</v>
       </c>
@@ -12534,12 +12956,16 @@
         <v>809</v>
       </c>
       <c r="L174" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M174" s="7"/>
       <c r="N174" s="2"/>
-      <c r="O174" s="2"/>
-      <c r="P174" s="2"/>
+      <c r="O174" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="P174" s="2" t="s">
+        <v>1155</v>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="K2:K168">
@@ -12744,7 +13170,9 @@
       </c>
     </row>
     <row r="3" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="2"/>
+      <c r="A3" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B3" s="2" t="s">
         <v>822</v>
       </c>
@@ -12782,12 +13210,16 @@
         <v>826</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="O3" s="7"/>
       <c r="P3" s="2"/>
-      <c r="Q3" s="2"/>
-      <c r="R3" s="2"/>
+      <c r="Q3" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="R3" s="2" t="s">
+        <v>1159</v>
+      </c>
     </row>
     <row r="4" spans="1:18" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
@@ -12844,7 +13276,9 @@
       </c>
     </row>
     <row r="5" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="2"/>
+      <c r="A5" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B5" s="2" t="s">
         <v>832</v>
       </c>
@@ -12882,15 +13316,21 @@
         <v>835</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="O5" s="7"/>
       <c r="P5" s="2"/>
-      <c r="Q5" s="2"/>
-      <c r="R5" s="2"/>
+      <c r="Q5" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="R5" s="2" t="s">
+        <v>1159</v>
+      </c>
     </row>
     <row r="6" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="2"/>
+      <c r="A6" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B6" s="2" t="s">
         <v>836</v>
       </c>
@@ -12928,12 +13368,16 @@
         <v>839</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="O6" s="7"/>
       <c r="P6" s="2"/>
-      <c r="Q6" s="2"/>
-      <c r="R6" s="2"/>
+      <c r="Q6" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="R6" s="2" t="s">
+        <v>1159</v>
+      </c>
     </row>
     <row r="7" spans="1:18" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
@@ -13152,7 +13596,9 @@
       </c>
     </row>
     <row r="11" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="2"/>
+      <c r="A11" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B11" s="2" t="s">
         <v>857</v>
       </c>
@@ -13190,15 +13636,21 @@
         <v>860</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="O11" s="7"/>
       <c r="P11" s="2"/>
-      <c r="Q11" s="2"/>
-      <c r="R11" s="2"/>
+      <c r="Q11" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="R11" s="2" t="s">
+        <v>1159</v>
+      </c>
     </row>
     <row r="12" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="2"/>
+      <c r="A12" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B12" s="2" t="s">
         <v>861</v>
       </c>
@@ -13236,15 +13688,21 @@
         <v>864</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="O12" s="7"/>
       <c r="P12" s="2"/>
-      <c r="Q12" s="2"/>
-      <c r="R12" s="2"/>
+      <c r="Q12" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="R12" s="2" t="s">
+        <v>1159</v>
+      </c>
     </row>
     <row r="13" spans="1:18" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="2"/>
+      <c r="A13" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B13" s="2" t="s">
         <v>865</v>
       </c>
@@ -13282,15 +13740,23 @@
         <v>868</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="O13" s="7"/>
+        <v>10</v>
+      </c>
+      <c r="O13" s="7">
+        <v>46324</v>
+      </c>
       <c r="P13" s="2"/>
-      <c r="Q13" s="2"/>
-      <c r="R13" s="2"/>
+      <c r="Q13" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="R13" s="2" t="s">
+        <v>1160</v>
+      </c>
     </row>
     <row r="14" spans="1:18" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="2"/>
+      <c r="A14" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B14" s="2" t="s">
         <v>869</v>
       </c>
@@ -13328,15 +13794,21 @@
         <v>875</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="O14" s="7"/>
       <c r="P14" s="2"/>
-      <c r="Q14" s="2"/>
-      <c r="R14" s="2"/>
+      <c r="Q14" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="R14" s="2" t="s">
+        <v>1159</v>
+      </c>
     </row>
     <row r="15" spans="1:18" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="2"/>
+      <c r="A15" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B15" s="2" t="s">
         <v>876</v>
       </c>
@@ -13374,12 +13846,16 @@
         <v>879</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="O15" s="7"/>
       <c r="P15" s="2"/>
-      <c r="Q15" s="2"/>
-      <c r="R15" s="2"/>
+      <c r="Q15" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="R15" s="2" t="s">
+        <v>1159</v>
+      </c>
     </row>
     <row r="16" spans="1:18" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
@@ -13428,7 +13904,9 @@
       <c r="R16" s="2"/>
     </row>
     <row r="17" spans="1:18" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="2"/>
+      <c r="A17" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B17" s="2" t="s">
         <v>884</v>
       </c>
@@ -13466,15 +13944,21 @@
         <v>887</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="O17" s="7"/>
       <c r="P17" s="2"/>
-      <c r="Q17" s="2"/>
-      <c r="R17" s="2"/>
+      <c r="Q17" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="R17" s="2" t="s">
+        <v>1159</v>
+      </c>
     </row>
     <row r="18" spans="1:18" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="2"/>
+      <c r="A18" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B18" s="2" t="s">
         <v>888</v>
       </c>
@@ -13512,12 +13996,16 @@
         <v>891</v>
       </c>
       <c r="N18" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="O18" s="7"/>
       <c r="P18" s="2"/>
-      <c r="Q18" s="2"/>
-      <c r="R18" s="2"/>
+      <c r="Q18" s="2" t="s">
+        <v>1157</v>
+      </c>
+      <c r="R18" s="2" t="s">
+        <v>1159</v>
+      </c>
     </row>
     <row r="19" spans="1:18" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
@@ -15223,7 +15711,9 @@
       </c>
     </row>
     <row r="3" spans="1:15" ht="105" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="2"/>
+      <c r="A3" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B3" s="2" t="s">
         <v>998</v>
       </c>
@@ -15249,18 +15739,24 @@
         <v>1003</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K3" s="7"/>
       <c r="L3" s="2"/>
-      <c r="M3" s="2"/>
+      <c r="M3" s="2" t="s">
+        <v>1157</v>
+      </c>
       <c r="N3" s="2" t="s">
         <v>1004</v>
       </c>
-      <c r="O3" s="2"/>
+      <c r="O3" s="2" t="s">
+        <v>1158</v>
+      </c>
     </row>
     <row r="4" spans="1:15" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2"/>
+      <c r="A4" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B4" s="2" t="s">
         <v>1005</v>
       </c>
@@ -15286,15 +15782,19 @@
         <v>1010</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K4" s="7"/>
       <c r="L4" s="2"/>
-      <c r="M4" s="2"/>
+      <c r="M4" s="2" t="s">
+        <v>1157</v>
+      </c>
       <c r="N4" s="2" t="s">
         <v>1004</v>
       </c>
-      <c r="O4" s="2"/>
+      <c r="O4" s="2" t="s">
+        <v>1158</v>
+      </c>
     </row>
     <row r="5" spans="1:15" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
@@ -15556,7 +16056,9 @@
       <c r="O11" s="2"/>
     </row>
     <row r="12" spans="1:15" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="2"/>
+      <c r="A12" s="2" t="s">
+        <v>1156</v>
+      </c>
       <c r="B12" s="2" t="s">
         <v>1052</v>
       </c>
@@ -15582,11 +16084,13 @@
         <v>1057</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K12" s="7"/>
       <c r="L12" s="2"/>
-      <c r="M12" s="2"/>
+      <c r="M12" s="2" t="s">
+        <v>1157</v>
+      </c>
       <c r="N12" s="2"/>
       <c r="O12" s="2" t="s">
         <v>1058</v>
@@ -15846,7 +16350,7 @@
       </c>
       <c r="J3" s="2" t="str">
         <f>IFERROR(INDEX('Security Acceptance'!$N:$N,MATCH($I3,'Security Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K3" s="7">
         <f>IFERROR(INDEX('Security Acceptance'!$O:$O,MATCH($I3,'Security Acceptance'!$B:$B,0)),"")</f>
@@ -15856,9 +16360,9 @@
         <f>IFERROR(INDEX('Security Acceptance'!$P:$P,MATCH($I3,'Security Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M3" s="2">
+      <c r="M3" s="2" t="str">
         <f>IFERROR(INDEX('Security Acceptance'!$Q:$Q,MATCH($I3,'Security Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N3" s="2" t="s">
         <v>1075</v>
@@ -15944,7 +16448,7 @@
       </c>
       <c r="J5" s="2" t="str">
         <f>IFERROR(INDEX('Security Acceptance'!$N:$N,MATCH($I5,'Security Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K5" s="7">
         <f>IFERROR(INDEX('Security Acceptance'!$O:$O,MATCH($I5,'Security Acceptance'!$B:$B,0)),"")</f>
@@ -15954,9 +16458,9 @@
         <f>IFERROR(INDEX('Security Acceptance'!$P:$P,MATCH($I5,'Security Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M5" s="2">
+      <c r="M5" s="2" t="str">
         <f>IFERROR(INDEX('Security Acceptance'!$Q:$Q,MATCH($I5,'Security Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N5" s="2" t="s">
         <v>1075</v>
@@ -15993,7 +16497,7 @@
       </c>
       <c r="J6" s="2" t="str">
         <f>IFERROR(INDEX('Security Acceptance'!$N:$N,MATCH($I6,'Security Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K6" s="7">
         <f>IFERROR(INDEX('Security Acceptance'!$O:$O,MATCH($I6,'Security Acceptance'!$B:$B,0)),"")</f>
@@ -16003,9 +16507,9 @@
         <f>IFERROR(INDEX('Security Acceptance'!$P:$P,MATCH($I6,'Security Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M6" s="2">
+      <c r="M6" s="2" t="str">
         <f>IFERROR(INDEX('Security Acceptance'!$Q:$Q,MATCH($I6,'Security Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N6" s="2" t="s">
         <v>1075</v>
@@ -16319,7 +16823,7 @@
       </c>
       <c r="J13" s="2" t="str">
         <f>IFERROR(INDEX('Security Acceptance'!$N:$N,MATCH($I13,'Security Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K13" s="7">
         <f>IFERROR(INDEX('Security Acceptance'!$O:$O,MATCH($I13,'Security Acceptance'!$B:$B,0)),"")</f>
@@ -16329,9 +16833,9 @@
         <f>IFERROR(INDEX('Security Acceptance'!$P:$P,MATCH($I13,'Security Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M13" s="2">
+      <c r="M13" s="2" t="str">
         <f>IFERROR(INDEX('Security Acceptance'!$Q:$Q,MATCH($I13,'Security Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N13" s="2" t="s">
         <v>1075</v>
@@ -16368,7 +16872,7 @@
       </c>
       <c r="J14" s="2" t="str">
         <f>IFERROR(INDEX('Security Acceptance'!$N:$N,MATCH($I14,'Security Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K14" s="7">
         <f>IFERROR(INDEX('Security Acceptance'!$O:$O,MATCH($I14,'Security Acceptance'!$B:$B,0)),"")</f>
@@ -16378,9 +16882,9 @@
         <f>IFERROR(INDEX('Security Acceptance'!$P:$P,MATCH($I14,'Security Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M14" s="2">
+      <c r="M14" s="2" t="str">
         <f>IFERROR(INDEX('Security Acceptance'!$Q:$Q,MATCH($I14,'Security Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N14" s="2" t="s">
         <v>1075</v>
@@ -16417,19 +16921,19 @@
       </c>
       <c r="J15" s="2" t="str">
         <f>IFERROR(INDEX('Security Acceptance'!$N:$N,MATCH($I15,'Security Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Pass</v>
       </c>
       <c r="K15" s="7">
         <f>IFERROR(INDEX('Security Acceptance'!$O:$O,MATCH($I15,'Security Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>46324</v>
       </c>
       <c r="L15" s="2">
         <f>IFERROR(INDEX('Security Acceptance'!$P:$P,MATCH($I15,'Security Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M15" s="2">
+      <c r="M15" s="2" t="str">
         <f>IFERROR(INDEX('Security Acceptance'!$Q:$Q,MATCH($I15,'Security Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N15" s="2" t="s">
         <v>1075</v>
@@ -16709,7 +17213,7 @@
       </c>
       <c r="J21" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I21,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K21" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I21,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -16719,9 +17223,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I21,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M21" s="2">
+      <c r="M21" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I21,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N21" s="2" t="s">
         <v>1075</v>
@@ -16758,7 +17262,7 @@
       </c>
       <c r="J22" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I22,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K22" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I22,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -16768,9 +17272,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I22,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M22" s="2">
+      <c r="M22" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I22,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N22" s="2" t="s">
         <v>1075</v>
@@ -16942,7 +17446,7 @@
       </c>
       <c r="J26" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I26,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K26" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I26,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -16952,9 +17456,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I26,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M26" s="2">
+      <c r="M26" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I26,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N26" s="2" t="s">
         <v>1075</v>
@@ -16991,7 +17495,7 @@
       </c>
       <c r="J27" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I27,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K27" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I27,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -17001,9 +17505,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I27,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M27" s="2">
+      <c r="M27" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I27,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N27" s="2" t="s">
         <v>1075</v>
@@ -17040,7 +17544,7 @@
       </c>
       <c r="J28" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I28,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K28" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I28,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -17050,9 +17554,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I28,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M28" s="2">
+      <c r="M28" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I28,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N28" s="2" t="s">
         <v>1075</v>
@@ -17089,7 +17593,7 @@
       </c>
       <c r="J29" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I29,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K29" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I29,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -17099,9 +17603,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I29,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M29" s="2">
+      <c r="M29" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I29,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N29" s="2" t="s">
         <v>1075</v>
@@ -17138,7 +17642,7 @@
       </c>
       <c r="J30" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I30,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K30" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I30,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -17148,9 +17652,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I30,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M30" s="2">
+      <c r="M30" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I30,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N30" s="2" t="s">
         <v>1075</v>
@@ -17187,7 +17691,7 @@
       </c>
       <c r="J31" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I31,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K31" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I31,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -17197,9 +17701,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I31,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M31" s="2">
+      <c r="M31" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I31,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N31" s="2" t="s">
         <v>1075</v>
@@ -17236,7 +17740,7 @@
       </c>
       <c r="J32" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I32,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K32" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I32,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -17246,9 +17750,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I32,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M32" s="2">
+      <c r="M32" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I32,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N32" s="2" t="s">
         <v>1075</v>
@@ -17285,7 +17789,7 @@
       </c>
       <c r="J33" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I33,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K33" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I33,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -17295,9 +17799,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I33,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M33" s="2">
+      <c r="M33" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I33,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N33" s="2" t="s">
         <v>1075</v>
@@ -17334,7 +17838,7 @@
       </c>
       <c r="J34" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I34,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K34" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I34,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -17344,9 +17848,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I34,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M34" s="2">
+      <c r="M34" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I34,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N34" s="2" t="s">
         <v>1075</v>
@@ -17383,7 +17887,7 @@
       </c>
       <c r="J35" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I35,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K35" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I35,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -17393,9 +17897,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I35,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M35" s="2">
+      <c r="M35" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I35,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N35" s="2" t="s">
         <v>1075</v>
@@ -17432,7 +17936,7 @@
       </c>
       <c r="J36" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I36,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K36" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I36,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -17442,9 +17946,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I36,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M36" s="2">
+      <c r="M36" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I36,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N36" s="2" t="s">
         <v>1075</v>
@@ -17481,7 +17985,7 @@
       </c>
       <c r="J37" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I37,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K37" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I37,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -17491,9 +17995,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I37,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M37" s="2">
+      <c r="M37" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I37,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N37" s="2" t="s">
         <v>1075</v>
@@ -17530,7 +18034,7 @@
       </c>
       <c r="J38" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I38,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K38" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I38,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -17540,9 +18044,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I38,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M38" s="2">
+      <c r="M38" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I38,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N38" s="2" t="s">
         <v>1075</v>
@@ -17579,7 +18083,7 @@
       </c>
       <c r="J39" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I39,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K39" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I39,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -17589,9 +18093,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I39,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M39" s="2">
+      <c r="M39" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I39,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N39" s="2" t="s">
         <v>1075</v>
@@ -17628,7 +18132,7 @@
       </c>
       <c r="J40" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I40,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K40" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I40,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -17638,9 +18142,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I40,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M40" s="2">
+      <c r="M40" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I40,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N40" s="2" t="s">
         <v>1075</v>
@@ -17824,7 +18328,7 @@
       </c>
       <c r="J44" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I44,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K44" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I44,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -17834,9 +18338,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I44,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M44" s="2">
+      <c r="M44" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I44,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N44" s="2" t="s">
         <v>1075</v>
@@ -17873,7 +18377,7 @@
       </c>
       <c r="J45" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I45,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K45" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I45,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -17883,9 +18387,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I45,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M45" s="2">
+      <c r="M45" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I45,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N45" s="2" t="s">
         <v>1075</v>
@@ -17922,7 +18426,7 @@
       </c>
       <c r="J46" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I46,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K46" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I46,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -17932,9 +18436,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I46,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M46" s="2">
+      <c r="M46" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I46,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N46" s="2" t="s">
         <v>1075</v>
@@ -17971,7 +18475,7 @@
       </c>
       <c r="J47" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I47,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K47" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I47,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -17981,9 +18485,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I47,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M47" s="2">
+      <c r="M47" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I47,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N47" s="2" t="s">
         <v>1075</v>
@@ -18020,7 +18524,7 @@
       </c>
       <c r="J48" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I48,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K48" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I48,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -18030,9 +18534,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I48,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M48" s="2">
+      <c r="M48" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I48,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N48" s="2" t="s">
         <v>1075</v>
@@ -18069,7 +18573,7 @@
       </c>
       <c r="J49" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I49,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K49" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I49,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -18079,9 +18583,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I49,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M49" s="2">
+      <c r="M49" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I49,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N49" s="2" t="s">
         <v>1075</v>
@@ -18167,7 +18671,7 @@
       </c>
       <c r="J51" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I51,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K51" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I51,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -18177,9 +18681,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I51,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M51" s="2">
+      <c r="M51" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I51,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N51" s="2" t="s">
         <v>1075</v>
@@ -18216,7 +18720,7 @@
       </c>
       <c r="J52" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I52,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K52" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I52,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -18226,9 +18730,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I52,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M52" s="2">
+      <c r="M52" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I52,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N52" s="2" t="s">
         <v>1075</v>
@@ -18265,7 +18769,7 @@
       </c>
       <c r="J53" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I53,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K53" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I53,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -18275,9 +18779,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I53,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M53" s="2">
+      <c r="M53" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I53,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N53" s="2" t="s">
         <v>1075</v>
@@ -18314,7 +18818,7 @@
       </c>
       <c r="J54" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I54,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K54" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I54,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -18324,9 +18828,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I54,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M54" s="2">
+      <c r="M54" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I54,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N54" s="2" t="s">
         <v>1075</v>
@@ -18461,7 +18965,7 @@
       </c>
       <c r="J57" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I57,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K57" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I57,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -18471,9 +18975,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I57,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M57" s="2">
+      <c r="M57" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I57,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N57" s="2" t="s">
         <v>1075</v>
@@ -18510,7 +19014,7 @@
       </c>
       <c r="J58" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I58,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K58" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I58,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -18520,9 +19024,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I58,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M58" s="2">
+      <c r="M58" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I58,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N58" s="2" t="s">
         <v>1075</v>
@@ -18559,7 +19063,7 @@
       </c>
       <c r="J59" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I59,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K59" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I59,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -18569,9 +19073,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I59,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M59" s="2">
+      <c r="M59" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I59,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N59" s="2" t="s">
         <v>1075</v>
@@ -18608,7 +19112,7 @@
       </c>
       <c r="J60" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I60,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K60" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I60,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -18618,9 +19122,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I60,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M60" s="2">
+      <c r="M60" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I60,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N60" s="2" t="s">
         <v>1075</v>
@@ -18755,7 +19259,7 @@
       </c>
       <c r="J63" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I63,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K63" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I63,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -18765,9 +19269,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I63,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M63" s="2">
+      <c r="M63" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I63,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N63" s="2" t="s">
         <v>1075</v>
@@ -18804,7 +19308,7 @@
       </c>
       <c r="J64" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I64,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K64" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I64,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -18814,9 +19318,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I64,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M64" s="2">
+      <c r="M64" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I64,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N64" s="2" t="s">
         <v>1075</v>
@@ -18853,7 +19357,7 @@
       </c>
       <c r="J65" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I65,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K65" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I65,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -18863,9 +19367,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I65,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M65" s="2">
+      <c r="M65" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I65,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N65" s="2" t="s">
         <v>1075</v>
@@ -18902,7 +19406,7 @@
       </c>
       <c r="J66" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I66,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K66" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I66,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -18912,9 +19416,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I66,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M66" s="2">
+      <c r="M66" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I66,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N66" s="2" t="s">
         <v>1075</v>
@@ -18951,7 +19455,7 @@
       </c>
       <c r="J67" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I67,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K67" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I67,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -18961,9 +19465,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I67,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M67" s="2">
+      <c r="M67" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I67,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N67" s="2" t="s">
         <v>1075</v>
@@ -19000,7 +19504,7 @@
       </c>
       <c r="J68" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I68,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K68" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I68,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -19010,9 +19514,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I68,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M68" s="2">
+      <c r="M68" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I68,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N68" s="2" t="s">
         <v>1075</v>
@@ -19049,7 +19553,7 @@
       </c>
       <c r="J69" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I69,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K69" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I69,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -19059,9 +19563,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I69,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M69" s="2">
+      <c r="M69" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I69,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N69" s="2" t="s">
         <v>1075</v>
@@ -19098,7 +19602,7 @@
       </c>
       <c r="J70" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I70,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K70" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I70,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -19108,9 +19612,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I70,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M70" s="2">
+      <c r="M70" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I70,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N70" s="2" t="s">
         <v>1075</v>
@@ -19147,7 +19651,7 @@
       </c>
       <c r="J71" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I71,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K71" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I71,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -19157,9 +19661,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I71,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M71" s="2">
+      <c r="M71" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I71,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N71" s="2" t="s">
         <v>1075</v>
@@ -19196,7 +19700,7 @@
       </c>
       <c r="J72" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I72,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K72" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I72,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -19206,9 +19710,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I72,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M72" s="2">
+      <c r="M72" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I72,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N72" s="2" t="s">
         <v>1075</v>
@@ -19245,7 +19749,7 @@
       </c>
       <c r="J73" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I73,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K73" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I73,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -19255,9 +19759,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I73,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M73" s="2">
+      <c r="M73" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I73,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N73" s="2" t="s">
         <v>1075</v>
@@ -19294,7 +19798,7 @@
       </c>
       <c r="J74" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I74,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K74" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I74,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -19304,9 +19808,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I74,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M74" s="2">
+      <c r="M74" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I74,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N74" s="2" t="s">
         <v>1075</v>
@@ -19343,7 +19847,7 @@
       </c>
       <c r="J75" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I75,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K75" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I75,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -19353,9 +19857,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I75,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M75" s="2">
+      <c r="M75" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I75,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N75" s="2" t="s">
         <v>1075</v>
@@ -19392,7 +19896,7 @@
       </c>
       <c r="J76" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I76,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K76" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I76,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -19402,9 +19906,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I76,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M76" s="2">
+      <c r="M76" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I76,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N76" s="2" t="s">
         <v>1075</v>
@@ -19441,7 +19945,7 @@
       </c>
       <c r="J77" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I77,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K77" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I77,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -19451,9 +19955,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I77,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M77" s="2">
+      <c r="M77" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I77,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N77" s="2" t="s">
         <v>1075</v>
@@ -19490,7 +19994,7 @@
       </c>
       <c r="J78" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I78,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K78" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I78,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -19500,9 +20004,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I78,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M78" s="2">
+      <c r="M78" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I78,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N78" s="2" t="s">
         <v>1075</v>
@@ -19539,7 +20043,7 @@
       </c>
       <c r="J79" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I79,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K79" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I79,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -19549,9 +20053,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I79,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M79" s="2">
+      <c r="M79" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I79,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N79" s="2" t="s">
         <v>1075</v>
@@ -19588,7 +20092,7 @@
       </c>
       <c r="J80" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I80,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K80" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I80,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -19598,9 +20102,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I80,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M80" s="2">
+      <c r="M80" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I80,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N80" s="2" t="s">
         <v>1075</v>
@@ -19637,7 +20141,7 @@
       </c>
       <c r="J81" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I81,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K81" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I81,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -19647,9 +20151,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I81,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M81" s="2">
+      <c r="M81" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I81,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N81" s="2" t="s">
         <v>1075</v>
@@ -19686,7 +20190,7 @@
       </c>
       <c r="J82" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I82,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K82" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I82,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -19696,9 +20200,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I82,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M82" s="2">
+      <c r="M82" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I82,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N82" s="2" t="s">
         <v>1075</v>
@@ -19735,7 +20239,7 @@
       </c>
       <c r="J83" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I83,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K83" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I83,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -19745,9 +20249,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I83,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M83" s="2">
+      <c r="M83" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I83,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N83" s="2" t="s">
         <v>1075</v>
@@ -19784,7 +20288,7 @@
       </c>
       <c r="J84" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I84,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K84" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I84,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -19794,9 +20298,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I84,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M84" s="2">
+      <c r="M84" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I84,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N84" s="2" t="s">
         <v>1075</v>
@@ -19833,7 +20337,7 @@
       </c>
       <c r="J85" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I85,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K85" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I85,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -19843,9 +20347,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I85,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M85" s="2">
+      <c r="M85" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I85,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N85" s="2" t="s">
         <v>1075</v>
@@ -19882,7 +20386,7 @@
       </c>
       <c r="J86" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I86,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K86" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I86,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -19892,9 +20396,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I86,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M86" s="2">
+      <c r="M86" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I86,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N86" s="2" t="s">
         <v>1075</v>
@@ -24292,7 +24796,7 @@
       </c>
       <c r="J176" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I176,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K176" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I176,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -24302,9 +24806,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I176,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M176" s="2">
+      <c r="M176" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I176,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N176" s="2" t="s">
         <v>1075</v>
@@ -24341,7 +24845,7 @@
       </c>
       <c r="J177" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I177,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K177" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I177,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -24351,9 +24855,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I177,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M177" s="2">
+      <c r="M177" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I177,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N177" s="2" t="s">
         <v>1075</v>
@@ -24390,7 +24894,7 @@
       </c>
       <c r="J178" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I178,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K178" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I178,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -24400,9 +24904,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I178,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M178" s="2">
+      <c r="M178" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I178,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N178" s="2" t="s">
         <v>1075</v>
@@ -24439,7 +24943,7 @@
       </c>
       <c r="J179" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I179,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K179" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I179,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -24449,9 +24953,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I179,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M179" s="2">
+      <c r="M179" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I179,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N179" s="2" t="s">
         <v>1075</v>
@@ -24488,7 +24992,7 @@
       </c>
       <c r="J180" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I180,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K180" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I180,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -24498,9 +25002,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I180,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M180" s="2">
+      <c r="M180" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I180,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N180" s="2" t="s">
         <v>1075</v>
@@ -24537,7 +25041,7 @@
       </c>
       <c r="J181" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I181,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K181" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I181,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -24547,9 +25051,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I181,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M181" s="2">
+      <c r="M181" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I181,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N181" s="2" t="s">
         <v>1075</v>
@@ -24586,7 +25090,7 @@
       </c>
       <c r="J182" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I182,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K182" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I182,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -24596,9 +25100,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I182,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M182" s="2">
+      <c r="M182" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I182,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N182" s="2" t="s">
         <v>1075</v>
@@ -24684,7 +25188,7 @@
       </c>
       <c r="J184" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I184,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K184" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I184,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -24694,9 +25198,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I184,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M184" s="2">
+      <c r="M184" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I184,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N184" s="2" t="s">
         <v>1075</v>
@@ -25331,7 +25835,7 @@
       </c>
       <c r="J198" s="2" t="str">
         <f>IFERROR(INDEX('Security Acceptance'!$N:$N,MATCH($I198,'Security Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K198" s="7">
         <f>IFERROR(INDEX('Security Acceptance'!$O:$O,MATCH($I198,'Security Acceptance'!$B:$B,0)),"")</f>
@@ -25341,9 +25845,9 @@
         <f>IFERROR(INDEX('Security Acceptance'!$P:$P,MATCH($I198,'Security Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M198" s="2">
+      <c r="M198" s="2" t="str">
         <f>IFERROR(INDEX('Security Acceptance'!$Q:$Q,MATCH($I198,'Security Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N198" s="2" t="s">
         <v>1075</v>
@@ -25380,7 +25884,7 @@
       </c>
       <c r="J199" s="2" t="str">
         <f>IFERROR(INDEX('Security Acceptance'!$N:$N,MATCH($I199,'Security Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K199" s="7">
         <f>IFERROR(INDEX('Security Acceptance'!$O:$O,MATCH($I199,'Security Acceptance'!$B:$B,0)),"")</f>
@@ -25390,9 +25894,9 @@
         <f>IFERROR(INDEX('Security Acceptance'!$P:$P,MATCH($I199,'Security Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M199" s="2">
+      <c r="M199" s="2" t="str">
         <f>IFERROR(INDEX('Security Acceptance'!$Q:$Q,MATCH($I199,'Security Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N199" s="2" t="s">
         <v>1075</v>
@@ -25478,7 +25982,7 @@
       </c>
       <c r="J201" s="2" t="str">
         <f>IFERROR(INDEX('Security Acceptance'!$N:$N,MATCH($I201,'Security Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K201" s="7">
         <f>IFERROR(INDEX('Security Acceptance'!$O:$O,MATCH($I201,'Security Acceptance'!$B:$B,0)),"")</f>
@@ -25488,9 +25992,9 @@
         <f>IFERROR(INDEX('Security Acceptance'!$P:$P,MATCH($I201,'Security Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M201" s="2">
+      <c r="M201" s="2" t="str">
         <f>IFERROR(INDEX('Security Acceptance'!$Q:$Q,MATCH($I201,'Security Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N201" s="2" t="s">
         <v>1075</v>
@@ -25527,7 +26031,7 @@
       </c>
       <c r="J202" s="2" t="str">
         <f>IFERROR(INDEX('Security Acceptance'!$N:$N,MATCH($I202,'Security Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K202" s="7">
         <f>IFERROR(INDEX('Security Acceptance'!$O:$O,MATCH($I202,'Security Acceptance'!$B:$B,0)),"")</f>
@@ -25537,9 +26041,9 @@
         <f>IFERROR(INDEX('Security Acceptance'!$P:$P,MATCH($I202,'Security Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M202" s="2">
+      <c r="M202" s="2" t="str">
         <f>IFERROR(INDEX('Security Acceptance'!$Q:$Q,MATCH($I202,'Security Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N202" s="2" t="s">
         <v>1075</v>
@@ -26191,7 +26695,7 @@
       </c>
       <c r="J218" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I218,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K218" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I218,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -26201,9 +26705,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I218,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M218" s="2">
+      <c r="M218" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I218,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N218" s="2" t="s">
         <v>1075</v>
@@ -26240,7 +26744,7 @@
       </c>
       <c r="J219" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I219,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K219" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I219,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -26250,9 +26754,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I219,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M219" s="2">
+      <c r="M219" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I219,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N219" s="2" t="s">
         <v>1075</v>
@@ -26289,7 +26793,7 @@
       </c>
       <c r="J220" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I220,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K220" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I220,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -26299,9 +26803,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I220,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M220" s="2">
+      <c r="M220" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I220,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N220" s="2" t="s">
         <v>1075</v>
@@ -26338,7 +26842,7 @@
       </c>
       <c r="J221" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I221,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K221" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I221,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -26348,9 +26852,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I221,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M221" s="2">
+      <c r="M221" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I221,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N221" s="2" t="s">
         <v>1075</v>
@@ -26436,7 +26940,7 @@
       </c>
       <c r="J223" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$L:$L,MATCH($I223,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>Not Built</v>
+        <v>Ready to Test</v>
       </c>
       <c r="K223" s="7">
         <f>IFERROR(INDEX('Functional Acceptance'!$M:$M,MATCH($I223,'Functional Acceptance'!$B:$B,0)),"")</f>
@@ -26446,9 +26950,9 @@
         <f>IFERROR(INDEX('Functional Acceptance'!$N:$N,MATCH($I223,'Functional Acceptance'!$B:$B,0)),"")</f>
         <v>0</v>
       </c>
-      <c r="M223" s="2">
+      <c r="M223" s="2" t="str">
         <f>IFERROR(INDEX('Functional Acceptance'!$O:$O,MATCH($I223,'Functional Acceptance'!$B:$B,0)),"")</f>
-        <v>0</v>
+        <v>P1-TECH-001; dev baseline 8645287; spec/meals/README.md#phase-1-technical-evidence-and-limitations; phase1-focused-tests.log; phase1-full-tests.log; phase1-build-inspection.json</v>
       </c>
       <c r="N223" s="2" t="s">
         <v>1075</v>

</xml_diff>